<commit_message>
Remove empty sheets from moving items list
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013CaYEKiKpF8mzXjGXmPx4U
</commit_message>
<xml_diff>
--- a/seznam_svrsku_A4.xlsx
+++ b/seznam_svrsku_A4.xlsx
@@ -7,8 +7,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'List1'!$3:$3</definedName>
@@ -1577,30 +1575,4 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>